<commit_message>
Added Assert and data Provider
</commit_message>
<xml_diff>
--- a/src/test/resources/data/Testdata.xlsx
+++ b/src/test/resources/data/Testdata.xlsx
@@ -239,6 +239,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -259,6 +260,7 @@
       <sz val="18"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -266,11 +268,13 @@
       <color rgb="FF00A933"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -315,40 +319,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -538,349 +546,349 @@
   <dimension ref="A1:N10"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="14.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="19.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="17.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="17"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="true" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="4" customFormat="true" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="0"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="1"/>
     </row>
-    <row r="2" s="4" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+    <row r="2" s="5" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="0"/>
+      <c r="N2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="17.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="7" t="n">
-        <v>770123456</v>
-      </c>
-      <c r="F3" s="8" t="n">
+      <c r="E3" s="8" t="n">
+        <v>77012345600</v>
+      </c>
+      <c r="F3" s="9" t="n">
         <v>35927</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="7" t="n">
-        <v>760987654</v>
-      </c>
-      <c r="F4" s="8" t="n">
+      <c r="E4" s="8" t="n">
+        <v>76098765400</v>
+      </c>
+      <c r="F4" s="9" t="n">
         <v>36853</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="7" t="n">
-        <v>781456239</v>
-      </c>
-      <c r="F5" s="8" t="n">
+      <c r="E5" s="8" t="n">
+        <v>78145623900</v>
+      </c>
+      <c r="F5" s="9" t="n">
         <v>36227</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+    <row r="6" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="7" t="n">
-        <v>795632148</v>
-      </c>
-      <c r="F6" s="8" t="n">
+      <c r="E6" s="8" t="n">
+        <v>79563214800</v>
+      </c>
+      <c r="F6" s="9" t="n">
         <v>35626</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="K6" s="7" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="7" t="n">
-        <v>702365498</v>
-      </c>
-      <c r="F7" s="8" t="n">
+      <c r="E7" s="8" t="n">
+        <v>70236549800</v>
+      </c>
+      <c r="F7" s="9" t="n">
         <v>37136</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="6" t="s">
+      <c r="K7" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="7" t="n">
-        <v>774589632</v>
-      </c>
-      <c r="F8" s="8" t="n">
+      <c r="E8" s="8" t="n">
+        <v>77458963200</v>
+      </c>
+      <c r="F8" s="9" t="n">
         <v>35083</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="K8" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="9" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="7" t="n">
-        <v>760214589</v>
-      </c>
-      <c r="F9" s="8" t="n">
+      <c r="E9" s="8" t="n">
+        <v>76021458900</v>
+      </c>
+      <c r="F9" s="9" t="n">
         <v>35976</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="33.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="7" t="n">
-        <v>789654123</v>
-      </c>
-      <c r="F10" s="8" t="n">
+      <c r="E10" s="8" t="n">
+        <v>78965412300</v>
+      </c>
+      <c r="F10" s="9" t="n">
         <v>37540</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="I10" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="J10" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="K10" s="7" t="s">
         <v>67</v>
       </c>
     </row>

</xml_diff>